<commit_message>
fix RegistrationFee/AnnualCourseFee / excel
</commit_message>
<xml_diff>
--- a/FekraHubAPI/Controllers/students.xlsx
+++ b/FekraHubAPI/Controllers/students.xlsx
@@ -1894,7 +1894,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB302"/>
+  <dimension ref="A1:Z302"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.5546875" style="5" customWidth="1"/>
@@ -1912,11 +1912,9 @@
     <col min="24" max="24" width="22.44140625" customWidth="1"/>
     <col min="25" max="25" width="22.109375" customWidth="1"/>
     <col min="26" max="26" width="13.77734375" style="8" customWidth="1"/>
-    <col min="27" max="27" width="16" customWidth="1"/>
-    <col min="28" max="28" width="21.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18">
+    <row r="1" spans="1:26" ht="18">
       <c r="A1" s="39"/>
       <c r="B1" s="40" t="s">
         <v>12</v>
@@ -1930,11 +1928,11 @@
       <c r="I1" s="41"/>
       <c r="J1" s="41"/>
       <c r="K1" s="41"/>
-      <c r="L1" s="41"/>
-      <c r="M1" s="41"/>
-      <c r="N1" s="42" t="s">
+      <c r="L1" s="42" t="s">
         <v>13</v>
       </c>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
       <c r="O1" s="42"/>
       <c r="P1" s="42"/>
       <c r="Q1" s="42"/>
@@ -1947,10 +1945,8 @@
       <c r="X1" s="42"/>
       <c r="Y1" s="42"/>
       <c r="Z1" s="42"/>
-      <c r="AA1" s="42"/>
-      <c r="AB1" s="42"/>
-    </row>
-    <row r="2" spans="1:28" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="2" spans="1:26" ht="20.399999999999999" customHeight="1">
       <c r="A2" s="39"/>
       <c r="B2" s="20" t="s">
         <v>22</v>
@@ -2028,7 +2024,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:26" ht="25.05" customHeight="1">
       <c r="A3" s="4">
         <v>1</v>
       </c>
@@ -2058,7 +2054,7 @@
       <c r="Y3" s="9"/>
       <c r="Z3" s="10"/>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:26" ht="25.05" customHeight="1">
       <c r="A4" s="4">
         <v>2</v>
       </c>
@@ -2088,7 +2084,7 @@
       <c r="Y4" s="9"/>
       <c r="Z4" s="10"/>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:26" ht="25.05" customHeight="1">
       <c r="A5" s="4">
         <v>3</v>
       </c>
@@ -2118,7 +2114,7 @@
       <c r="Y5" s="9"/>
       <c r="Z5" s="10"/>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:26" ht="25.05" customHeight="1">
       <c r="A6" s="4">
         <v>4</v>
       </c>
@@ -2148,7 +2144,7 @@
       <c r="Y6" s="9"/>
       <c r="Z6" s="10"/>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:26" ht="25.05" customHeight="1">
       <c r="A7" s="4">
         <v>5</v>
       </c>
@@ -2178,7 +2174,7 @@
       <c r="Y7" s="9"/>
       <c r="Z7" s="10"/>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+    <row r="8" spans="1:26" ht="25.05" customHeight="1">
       <c r="A8" s="4">
         <v>6</v>
       </c>
@@ -2208,7 +2204,7 @@
       <c r="Y8" s="9"/>
       <c r="Z8" s="10"/>
     </row>
-    <row r="9" spans="1:28" ht="25.05" customHeight="1">
+    <row r="9" spans="1:26" ht="25.05" customHeight="1">
       <c r="A9" s="4">
         <v>7</v>
       </c>
@@ -2238,7 +2234,7 @@
       <c r="Y9" s="9"/>
       <c r="Z9" s="10"/>
     </row>
-    <row r="10" spans="1:28" ht="25.05" customHeight="1">
+    <row r="10" spans="1:26" ht="25.05" customHeight="1">
       <c r="A10" s="4">
         <v>8</v>
       </c>
@@ -2268,7 +2264,7 @@
       <c r="Y10" s="9"/>
       <c r="Z10" s="10"/>
     </row>
-    <row r="11" spans="1:28" ht="25.05" customHeight="1">
+    <row r="11" spans="1:26" ht="25.05" customHeight="1">
       <c r="A11" s="4">
         <v>9</v>
       </c>
@@ -2298,7 +2294,7 @@
       <c r="Y11" s="9"/>
       <c r="Z11" s="10"/>
     </row>
-    <row r="12" spans="1:28" ht="25.05" customHeight="1">
+    <row r="12" spans="1:26" ht="25.05" customHeight="1">
       <c r="A12" s="4">
         <v>10</v>
       </c>
@@ -2328,7 +2324,7 @@
       <c r="Y12" s="9"/>
       <c r="Z12" s="10"/>
     </row>
-    <row r="13" spans="1:28" ht="25.05" customHeight="1">
+    <row r="13" spans="1:26" ht="25.05" customHeight="1">
       <c r="A13" s="4">
         <v>11</v>
       </c>
@@ -2358,7 +2354,7 @@
       <c r="Y13" s="9"/>
       <c r="Z13" s="10"/>
     </row>
-    <row r="14" spans="1:28" ht="25.05" customHeight="1">
+    <row r="14" spans="1:26" ht="25.05" customHeight="1">
       <c r="A14" s="4">
         <v>12</v>
       </c>
@@ -2388,7 +2384,7 @@
       <c r="Y14" s="9"/>
       <c r="Z14" s="10"/>
     </row>
-    <row r="15" spans="1:28" ht="25.05" customHeight="1">
+    <row r="15" spans="1:26" ht="25.05" customHeight="1">
       <c r="A15" s="4">
         <v>13</v>
       </c>
@@ -2418,7 +2414,7 @@
       <c r="Y15" s="9"/>
       <c r="Z15" s="10"/>
     </row>
-    <row r="16" spans="1:28" ht="25.05" customHeight="1">
+    <row r="16" spans="1:26" ht="25.05" customHeight="1">
       <c r="A16" s="4">
         <v>14</v>
       </c>
@@ -11030,9 +11026,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="L1:Z1"/>
     <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:M1"/>
-    <mergeCell ref="N1:AB1"/>
+    <mergeCell ref="B1:K1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T3:T302 F3:F302">

</xml_diff>